<commit_message>
kurierebis 1% calke sheet mivamate
</commit_message>
<xml_diff>
--- a/output.xlsx
+++ b/output.xlsx
@@ -8,25 +8,26 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\nana\bank-summary\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D494672D-2C15-4AC0-AC38-F1225824DEF3}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="37" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6167C6E-AD17-47CB-A5F6-1D073B71016A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="37" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6816" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6816" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Results" sheetId="1" r:id="rId1"/>
     <sheet name="Summary" sheetId="2" r:id="rId2"/>
-    <sheet name="Salary" sheetId="3" r:id="rId3"/>
-    <sheet name="მომსახ დელ" sheetId="4" r:id="rId4"/>
-    <sheet name="მომსახ ცელ" sheetId="5" r:id="rId5"/>
-    <sheet name="ზუკა" sheetId="6" r:id="rId6"/>
-    <sheet name="ირმა" sheetId="7" r:id="rId7"/>
+    <sheet name="დელივერერები 1%" sheetId="8" r:id="rId3"/>
+    <sheet name="Salary" sheetId="3" r:id="rId4"/>
+    <sheet name="მომსახ დელ" sheetId="4" r:id="rId5"/>
+    <sheet name="მომსახ ცელ" sheetId="5" r:id="rId6"/>
+    <sheet name="ზუკა" sheetId="6" r:id="rId7"/>
+    <sheet name="ირმა" sheetId="7" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="39">
   <si>
     <t>Bank</t>
   </si>
@@ -153,7 +154,7 @@
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -193,6 +194,12 @@
       <color indexed="8"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="9">
@@ -258,7 +265,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -271,6 +278,9 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="43" fontId="0" fillId="7" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -926,7 +936,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -935,7 +945,7 @@
     <col min="4" max="4" width="49" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -949,7 +959,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" s="9" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="8" t="s">
         <v>11</v>
       </c>
@@ -962,8 +972,12 @@
       <c r="D2" s="8" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F2" s="12">
+        <f>C2*0.01</f>
+        <v>81.7667</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>25</v>
       </c>
@@ -979,8 +993,12 @@
       <c r="E3" s="2" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="F3" s="12">
+        <f t="shared" ref="F3:F13" si="0">C3*0.01</f>
+        <v>66.358400000000003</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" s="9" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A4" s="8" t="s">
         <v>11</v>
       </c>
@@ -993,8 +1011,12 @@
       <c r="D4" s="8" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="F4" s="12">
+        <f t="shared" si="0"/>
+        <v>61.235500000000002</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" s="9" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A5" s="8" t="s">
         <v>25</v>
       </c>
@@ -1007,8 +1029,12 @@
       <c r="D5" s="8" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="F5" s="12">
+        <f t="shared" si="0"/>
+        <v>55.346900000000012</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" s="9" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A6" s="8" t="s">
         <v>11</v>
       </c>
@@ -1021,8 +1047,12 @@
       <c r="D6" s="8" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F6" s="12">
+        <f t="shared" si="0"/>
+        <v>48.268899999999995</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>11</v>
       </c>
@@ -1038,8 +1068,12 @@
       <c r="E7" s="2" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="F7" s="12">
+        <f t="shared" si="0"/>
+        <v>47.329700000000003</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" s="9" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="8" t="s">
         <v>25</v>
       </c>
@@ -1052,8 +1086,12 @@
       <c r="D8" s="8" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="F8" s="12">
+        <f t="shared" si="0"/>
+        <v>43.064799999999998</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" s="9" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" s="8" t="s">
         <v>11</v>
       </c>
@@ -1066,8 +1104,12 @@
       <c r="D9" s="8" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="F9" s="12">
+        <f t="shared" si="0"/>
+        <v>41.856099999999998</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" s="9" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A10" s="8" t="s">
         <v>11</v>
       </c>
@@ -1080,8 +1122,12 @@
       <c r="D10" s="8" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="F10" s="12">
+        <f t="shared" si="0"/>
+        <v>33.050600000000003</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" s="9" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A11" s="8" t="s">
         <v>11</v>
       </c>
@@ -1094,8 +1140,12 @@
       <c r="D11" s="8" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F11" s="12">
+        <f t="shared" si="0"/>
+        <v>29.620100000000004</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>4</v>
       </c>
@@ -1108,8 +1158,12 @@
       <c r="D12" s="2" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="F12" s="12">
+        <f t="shared" si="0"/>
+        <v>9.7029999999999994</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" s="9" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A13" s="8" t="s">
         <v>11</v>
       </c>
@@ -1122,8 +1176,12 @@
       <c r="D13" s="8" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F13" s="12">
+        <f t="shared" si="0"/>
+        <v>5.6046000000000005</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="3"/>
       <c r="B14" s="3" t="s">
         <v>28</v>
@@ -1140,6 +1198,116 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{954EBA50-267C-45AD-A357-6C9100E13950}">
+  <dimension ref="B3:C14"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="22.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.88671875" style="14"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B3" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="14">
+        <v>81.7667</v>
+      </c>
+    </row>
+    <row r="4" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B4" s="13" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="14">
+        <v>66.358400000000003</v>
+      </c>
+    </row>
+    <row r="5" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B5" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" s="14">
+        <v>61.235500000000002</v>
+      </c>
+    </row>
+    <row r="6" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B6" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" s="14">
+        <v>55.346900000000012</v>
+      </c>
+    </row>
+    <row r="7" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B7" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7" s="14">
+        <v>48.268899999999995</v>
+      </c>
+    </row>
+    <row r="8" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B8" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" s="14">
+        <v>47.329700000000003</v>
+      </c>
+    </row>
+    <row r="9" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B9" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9" s="14">
+        <v>43.064799999999998</v>
+      </c>
+    </row>
+    <row r="10" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B10" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="C10" s="14">
+        <v>41.856099999999998</v>
+      </c>
+    </row>
+    <row r="11" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B11" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="C11" s="14">
+        <v>33.050600000000003</v>
+      </c>
+    </row>
+    <row r="12" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B12" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="C12" s="14">
+        <v>29.620100000000004</v>
+      </c>
+    </row>
+    <row r="13" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B13" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="C13" s="14">
+        <v>9.7029999999999994</v>
+      </c>
+    </row>
+    <row r="14" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B14" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="C14" s="14">
+        <v>5.6046000000000005</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:F15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1406,7 +1574,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:D14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1614,7 +1782,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1724,7 +1892,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1784,7 +1952,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>